<commit_message>
He añadido los resultados de los boxplots de yap/taz rankeando las drogas teniendo en cuanta la concentracion y mirando por tipo de tumor primario
</commit_message>
<xml_diff>
--- a/TFM_mao/resultados/technical_batch/anova_concentration.xlsx
+++ b/TFM_mao/resultados/technical_batch/anova_concentration.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>P_adj</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Veredicto</t>
         </is>
       </c>
@@ -462,7 +467,10 @@
       <c r="C2" t="n">
         <v>0.4307425233103424</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -480,7 +488,10 @@
       <c r="C3" t="n">
         <v>0.8864227677001011</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -498,7 +509,10 @@
       <c r="C4" t="n">
         <v>0.97991643393034</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -516,7 +530,10 @@
       <c r="C5" t="n">
         <v>0.7459016221665231</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -534,7 +551,10 @@
       <c r="C6" t="n">
         <v>0.9702613719217205</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -552,7 +572,10 @@
       <c r="C7" t="n">
         <v>0.9906347923444707</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -570,7 +593,10 @@
       <c r="C8" t="n">
         <v>0.9142024553256884</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -588,7 +614,10 @@
       <c r="C9" t="n">
         <v>0.9527914687348733</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -606,7 +635,10 @@
       <c r="C10" t="n">
         <v>0.9477263942219222</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -624,7 +656,10 @@
       <c r="C11" t="n">
         <v>0.9474964937149729</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -642,7 +677,10 @@
       <c r="C12" t="n">
         <v>0.7895112628876239</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -660,7 +698,10 @@
       <c r="C13" t="n">
         <v>0.6605031094878251</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -678,7 +719,10 @@
       <c r="C14" t="n">
         <v>0.8360408301135759</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -696,7 +740,10 @@
       <c r="C15" t="n">
         <v>0.8454197335138979</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -714,7 +761,10 @@
       <c r="C16" t="n">
         <v>0.7996032649749575</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -732,7 +782,10 @@
       <c r="C17" t="n">
         <v>0.4569282734675113</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -750,7 +803,10 @@
       <c r="C18" t="n">
         <v>0.7995147366522928</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -768,7 +824,10 @@
       <c r="C19" t="n">
         <v>0.5825819846152795</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -786,7 +845,10 @@
       <c r="C20" t="n">
         <v>0.881497514543125</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -804,7 +866,10 @@
       <c r="C21" t="n">
         <v>0.9564285848154223</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -822,7 +887,10 @@
       <c r="C22" t="n">
         <v>0.9125726707626935</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -840,7 +908,10 @@
       <c r="C23" t="n">
         <v>0.7440639085799668</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -858,7 +929,10 @@
       <c r="C24" t="n">
         <v>0.4320938619678146</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -876,7 +950,10 @@
       <c r="C25" t="n">
         <v>0.7563481100283918</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -894,7 +971,10 @@
       <c r="C26" t="n">
         <v>0.955180639146378</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -912,7 +992,10 @@
       <c r="C27" t="n">
         <v>0.2063021004144528</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -930,9 +1013,12 @@
       <c r="C28" t="n">
         <v>0.04225608672528403</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Significativo</t>
+      <c r="D28" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>No significativo</t>
         </is>
       </c>
     </row>
@@ -948,7 +1034,10 @@
       <c r="C29" t="n">
         <v>0.407922252557419</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -966,7 +1055,10 @@
       <c r="C30" t="n">
         <v>0.9882631586624562</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>
@@ -984,7 +1076,10 @@
       <c r="C31" t="n">
         <v>0.8472403384590602</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="n">
+        <v>0.9906347923444707</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>No significativo</t>
         </is>

</xml_diff>